<commit_message>
fundraising-cup: refresh deck + workbook with diversified article titles
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/fundraising-cup/keyword-research.xlsx
+++ b/decks/fundraising-cup/keyword-research.xlsx
@@ -632,7 +632,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Raffle Ideas: Inspiration for Your Next Campaign</t>
+          <t>Raffle Ideas Worth Trying</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Sample Nonprofit Bylaws, Explained</t>
+          <t>The Simple Guide to Sample Nonprofit Bylaws</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -852,7 +852,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>A Closer Look at Nonprofit Marketing</t>
+          <t>Nonprofit Marketing, Explained</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Understanding Donor Thank-You Letter</t>
+          <t>Donor Thank-You Letter, Demystified</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Nonprofit Marketing Plan: The Essentials</t>
+          <t>Understanding Nonprofit Marketing Plan</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1204,7 +1204,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>A Closer Look at Nonprofit Donation Form</t>
+          <t>The Simple Guide to Nonprofit Donation Form</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Peer to Peer Fundraising Platforms: A Field Guide</t>
+          <t>Choosing the Right Peer-to-Peer Fundraising Platforms</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Fundraising Gala: Where to Begin</t>
+          <t>Fundraising Gala: Start Here</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -1336,7 +1336,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Nonprofit Names: What to Know Before You Start</t>
+          <t>The Basics of Nonprofit Names</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1380,7 +1380,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Nonprofit Branding Strategy: A Complete Guide</t>
+          <t>Nonprofit Branding Strategy: What to Know Before You Start</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Nonprofit Branding, Explained</t>
+          <t>The Beginner's Guide to Nonprofit Branding</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -1468,7 +1468,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nonprofit Website Examples: Ideas That Actually Work</t>
+          <t>Nonprofit Website Examples, Step by Step</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Donor Thank-You Card: What to Know Before You Start</t>
+          <t>Everything to Know About Donor Thank-You Card</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Creative Takes on Donor Thank-You Letter Template</t>
+          <t>Donor Thank-You Letter Template: A Roundup Worth Bookmarking</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>The Not-for-Profit Business Plan, Explained</t>
+          <t>Building a Not-for-Profit Business Plan</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Gala Ball: Where to Begin</t>
+          <t>A Closer Look at Gala Ball</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Nonprofit Marketing Software: Getting It Right</t>
+          <t>Nonprofit Marketing Software: What to Expect</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Gala Program: A Practical Overview</t>
+          <t>Gala Program: What to Know Before You Start</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Best Nonprofit Website Design: What to Expect</t>
+          <t>Best Nonprofit Website Design, Done Right</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1908,7 +1908,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Donor Engagement Strategies: A Practical Overview</t>
+          <t>Donor Engagement Strategies: A Plain-English Guide</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -2040,7 +2040,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Gala Ideas: Inspiration for Your Next Campaign</t>
+          <t>Gala Ideas That Raise Real Money</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Spring Raffle Basket Ideas: A Side-by-Side Look</t>
+          <t>Spring Raffle Basket Ideas: From Idea to Impact</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -2172,7 +2172,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>School Raffle Basket Ideas: What Works Best</t>
+          <t>Smart School Raffle Basket Ideas for Any Cause</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2260,7 +2260,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Nonprofit Marketing Support: The Essentials</t>
+          <t>A Closer Look at Nonprofit Marketing Support</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -2304,7 +2304,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Peer to Peer Fundraising Examples: A Field Guide</t>
+          <t>Peer-to-Peer Fundraising Examples: Ideas That Actually Work</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Peer to Peer Fundraising Definition: A Field Guide</t>
+          <t>Peer-to-Peer Fundraising Definition: A Practical Overview</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -2524,7 +2524,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Peer-to-Peer Fundraising, Explained</t>
+          <t>How Peer-to-Peer Fundraising Works</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -2788,7 +2788,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Understanding Grant Money for Nonprofit</t>
+          <t>Grant Money for Nonprofit, Explained</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -2832,7 +2832,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Gala Themes: What to Know Before You Start</t>
+          <t>Gala Themes: Where to Begin</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -2876,7 +2876,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Ideas for Silent Auction Baskets: A Roundup Worth Bookmarking</t>
+          <t>Smart Ideas for Silent Auction Baskets for Any Cause</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Nonprofit Email Marketing: A Side-by-Side Look</t>
+          <t>Nonprofit Email Marketing: Inspiration for Your Next Campaign</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -3096,7 +3096,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Understanding Silent Auction Suggestions</t>
+          <t>Everything to Know About Silent Auction Suggestions</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Not-for-Profit Firms: The Essentials</t>
+          <t>Not-for-Profit Firms: Start Here</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -3184,7 +3184,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>A Closer Look at Silent Auction Items</t>
+          <t>Understanding Silent Auction Items</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Raffle Gift Ideas: What Works Best</t>
+          <t>Raffle Gift Ideas That Raise Real Money</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -3316,7 +3316,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Not-for-Profit Organization Example: Ideas That Actually Work</t>
+          <t>Not-for-Profit Organization Example: Lessons From Top Fundraisers</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -3360,7 +3360,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Understanding Nonprofit Social Media Strategy</t>
+          <t>Nonprofit Social Media Strategy: A Practical Overview</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -3404,7 +3404,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Cool Raffle Prizes, Explained</t>
+          <t>Cool Raffle Prizes: The Essentials</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -3448,7 +3448,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Not-for-Profit Advertising: A Roundup Worth Bookmarking</t>
+          <t>Not-for-Profit Advertising Worth Trying</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -3492,7 +3492,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>The Beginner's Guide to Donor Retention Rate</t>
+          <t>The Basics of Donor Retention Rate</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -3536,7 +3536,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>College Nonprofit Ideas, Step by Step</t>
+          <t>College Nonprofit Ideas: A Side-by-Side Look</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -3580,7 +3580,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>501c Types: The Essentials</t>
+          <t>501c Types, Demystified</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Nonprofit Marketing Plan Template: A Roundup Worth Bookmarking</t>
+          <t>Nonprofit Marketing Plan Template: What Works Best</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>A Closer Look at Nonprofit Storytelling</t>
+          <t>Nonprofit Storytelling: The Essentials</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -3712,7 +3712,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Choosing the Right Cool Nonprofit Websites</t>
+          <t>Picking the Best Cool Nonprofit Websites</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -3756,7 +3756,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Nonprofit Start Up Grants: Ideas That Actually Work</t>
+          <t>Nonprofit Start Up Grants That Raise Real Money</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Peer to Peer Fundraising Software: A Field Guide</t>
+          <t>Peer-to-Peer Fundraising Software: What to Look For</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -3844,7 +3844,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Gala Invitations: Proven Approaches</t>
+          <t>Gala Invitations: From Idea to Impact</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -3888,7 +3888,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Free Grant Database for Nonprofits: What to Look For</t>
+          <t>Free Grant Database for Nonprofits: A Practical Checklist</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -3932,7 +3932,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>P2P Fundraising Software: A Practical Checklist</t>
+          <t>P2P Fundraising Software: Getting It Right</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Peer to Peer Fundraising Nonprofits: A Field Guide</t>
+          <t>Peer-to-Peer Fundraising Nonprofits: Where to Begin</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Peer to Peer Fundraising Campaigns: A Field Guide</t>
+          <t>Peer-to-Peer Fundraising Campaigns, Explained</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Peer to Peer Fundraising Tips: A Field Guide</t>
+          <t>Creative Takes on Peer-to-Peer Fundraising Tips</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -4152,7 +4152,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Raffle Basket Ideas: Proven Approaches</t>
+          <t>Raffle Basket Ideas: Lessons From Top Fundraisers</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -4372,7 +4372,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Gala Event: Proven Approaches</t>
+          <t>Creative Takes on Gala Event</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -4504,7 +4504,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>The Beginner's Guide to Charity Gala</t>
+          <t>A Closer Look at Charity Gala</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -4636,7 +4636,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Raffle Fundraiser: A Complete Guide</t>
+          <t>Raffle Fundraiser: Start Here</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -4724,7 +4724,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Raffle Basket Ideas for Fundraiser, Step by Step</t>
+          <t>Raffle Basket Ideas for Fundraiser: From Idea to Impact</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -4768,7 +4768,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Nonprofit Christian Organizations: Where to Begin</t>
+          <t>Nonprofit Christian Organizations: A Complete Guide</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -4856,7 +4856,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Gala Invitation: Inspiration for Your Next Campaign</t>
+          <t>Gala Invitation: Tips From the Field</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
@@ -4900,7 +4900,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Gala Party: A Practical Overview</t>
+          <t>Gala Party: The Essentials</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -4944,7 +4944,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>The Beginner's Guide to Raffle Ticket Generator</t>
+          <t>Raffle Ticket Generator: What to Know Before You Start</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -5076,7 +5076,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Creative Takes on Silent Auction Bid Sheet Templates</t>
+          <t>Smart Silent Auction Bid Sheet Templates for Any Cause</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -5164,7 +5164,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>A Guide to Silent Auction Software</t>
+          <t>Picking the Best Silent Auction Software</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -5208,7 +5208,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Casino Gala: What to Know Before You Start</t>
+          <t>Understanding Casino Gala</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -5252,7 +5252,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Raffle Gift Certificate, Explained</t>
+          <t>Raffle Gift Certificate, Demystified</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
@@ -5340,7 +5340,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Understanding Online Silent Auction</t>
+          <t>Online Silent Auction: Start Here</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -5428,7 +5428,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Paypal for Nonprofit Organization: Where to Begin</t>
+          <t>A Guide to Paypal for Nonprofit Organization</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
@@ -5472,7 +5472,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>A Guide to Silent Auction Rules</t>
+          <t>Everything to Know About Silent Auction Rules</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -5516,7 +5516,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Raffle Suggestions: What to Know Before You Start</t>
+          <t>Raffle Suggestions, Demystified</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
@@ -5560,7 +5560,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Suggestions for Raffle Prizes: A Practical Overview</t>
+          <t>The Basics of Suggestions for Raffle Prizes</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -5604,7 +5604,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>A Guide to Silent Auction Template</t>
+          <t>Smart Silent Auction Template for Any Cause</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
@@ -5648,7 +5648,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Creative Takes on Fundraising Ideas for Nonprofit Organisations</t>
+          <t>Fundraising Ideas for Nonprofit Organisations: Lessons From Top Fundraisers</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
@@ -5692,7 +5692,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Nonprofit Churches: Tips From the Field</t>
+          <t>Nonprofit Churches: Proven Approaches</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
@@ -5736,7 +5736,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Nonprofit Fundraising Events, Explained</t>
+          <t>The Basics of Nonprofit Fundraising Events</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -5780,7 +5780,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Christmas Raffle: Tips From the Field</t>
+          <t>Christmas Raffle Worth Trying</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -5824,7 +5824,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>501c Organizations List: A Complete Guide</t>
+          <t>Everything to Know About 501c Organizations List</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">

</xml_diff>

<commit_message>
fundraising-cup: title grammar fix refresh
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/decks/fundraising-cup/keyword-research.xlsx
+++ b/decks/fundraising-cup/keyword-research.xlsx
@@ -616,7 +616,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Popcorn Fundraiser That Raise Real Money</t>
+          <t>Popcorn Fundraisers: How They Work + Best Companies</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Silent Auction Bid Sheet Template: Proven Approaches</t>
+          <t>Silent Auction Bid Sheet Template: A Roundup Worth Bookmarking</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Donation Receipt Template: From Idea to Impact</t>
+          <t>Donation Receipt Template Worth Trying</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -924,7 +924,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Online Fundraisers: Inspiration for Your Next Campaign</t>
+          <t>Online Fundraisers: Ideas That Actually Work</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Creative Takes on Sports Fundraising Ideas</t>
+          <t>Sports Fundraising Ideas, Step by Step</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1056,7 +1056,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Fundraising Ideas for Sports Teams: Tips From the Field</t>
+          <t>Creative Takes on Fundraising Ideas for Sports Teams</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>High School Fundraising Ideas: Tips From the Field</t>
+          <t>Creative Takes on High School Fundraising Ideas</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -1320,7 +1320,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Football Fundraising Ideas: A Side-by-Side Look</t>
+          <t>Football Fundraising Ideas: What Works Best</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -1496,7 +1496,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Christmas Fundraising Ideas Worth Trying</t>
+          <t>Christmas Fundraising Ideas: Lessons From Top Fundraisers</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -1540,7 +1540,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Fundraising Ideas for School Clubs: A Side-by-Side Look</t>
+          <t>Fundraising Ideas for School Clubs: Tips From the Field</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Smart Baseball Fundraising Ideas for Any Cause</t>
+          <t>Baseball Fundraising Ideas: Tips From the Field</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
@@ -1628,7 +1628,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Softball Fundraiser Ideas: Lessons From Top Fundraisers</t>
+          <t>Softball Fundraiser Ideas: A Side-by-Side Look</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Ideas for Fundraising for Individuals, Step by Step</t>
+          <t>Ideas for Fundraising for Individuals: Proven Approaches</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Donation Form Template: From Idea to Impact</t>
+          <t>Donation Form Template: Lessons From Top Fundraisers</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -1936,7 +1936,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Donor Gifts That Raise Real Money</t>
+          <t>Donor Gifts Worth Trying</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -2156,7 +2156,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Fundraising Plan Template That Raise Real Money</t>
+          <t>Fundraising Plan Templates: A Practical Starter</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>School Fundraising Ideas, Step by Step</t>
+          <t>School Fundraising Ideas: Inspiration for Your Next Campaign</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -2552,7 +2552,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Fundraising Ideas for Schools: What Works Best</t>
+          <t>Fundraising Ideas for Schools, Step by Step</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2684,7 +2684,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Raise Funds Ideas: A Roundup Worth Bookmarking</t>
+          <t>Raise Funds Ideas: From Idea to Impact</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Silent Auction Basket Ideas: Inspiration for Your Next Campaign</t>
+          <t>Silent Auction Basket Ideas: Proven Approaches</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Church Fundraiser Ideas: Proven Approaches</t>
+          <t>Church Fundraiser Ideas: A Roundup Worth Bookmarking</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -2992,7 +2992,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Gala Event: Ideas That Actually Work</t>
+          <t>Gala Event: From Idea to Impact</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -3080,7 +3080,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Creative Takes on Fundraising Ideas for Students</t>
+          <t>Fundraising Ideas for Students: What Works Best</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Ways to Give: Lessons From Top Fundraisers</t>
+          <t>Smart Ways to Give for Any Cause</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -3564,7 +3564,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Smart PTO Fundraising Ideas for Any Cause</t>
+          <t>PTO Fundraising Ideas: A Side-by-Side Look</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -5148,7 +5148,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Grant County Humane Society Worth Trying</t>
+          <t>Smart Grant County Humane Society for Any Cause</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Candy Fundraiser: Ideas That Actually Work</t>
+          <t>Candy Fundraiser: A Proven Money-Maker</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Crowdfunding for My Business: What Works Best</t>
+          <t>Crowdfunding for My Business: Inspiration for Your Next Campaign</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -5764,7 +5764,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Letter Asking for Donations Template: Ideas That Actually Work</t>
+          <t>Letter Asking for Donations Template: A Proven Money-Maker</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -5808,7 +5808,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Product Fundraising: A Roundup Worth Bookmarking</t>
+          <t>Product Fundraising: Ideas That Actually Work</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">

</xml_diff>